<commit_message>
Update FundFlow ETL pipeline and dashboard
</commit_message>
<xml_diff>
--- a/reports/global_mutual_fund_source_inventory.xlsx
+++ b/reports/global_mutual_fund_source_inventory.xlsx
@@ -18,12 +18,12 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dashboard'!$A$1:$B$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Asia-Pacific'!$A$1:$AI$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Europe'!$A$1:$AI$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'North America'!$A$1:$AI$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Asia-Pacific'!$A$1:$AI$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Europe'!$A$1:$AI$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'North America'!$A$1:$AI$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Other Markets'!$A$1:$AI$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Source Verification Log'!$A$1:$I$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'ETL Integration Status'!$A$1:$H$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'ETL Integration Status'!$A$1:$H$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Data Dictionary'!$A$1:$B$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -326,8 +326,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Asia-PacificSources" displayName="Asia-PacificSources" ref="A1:AI9" headerRowCount="1">
-  <autoFilter ref="A1:AI9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Asia-PacificSources" displayName="Asia-PacificSources" ref="A1:AI10" headerRowCount="1">
+  <autoFilter ref="A1:AI10"/>
   <tableColumns count="35">
     <tableColumn id="1" name="Source ID"/>
     <tableColumn id="2" name="Country"/>
@@ -370,8 +370,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EuropeSources" displayName="EuropeSources" ref="A1:AI15" headerRowCount="1">
-  <autoFilter ref="A1:AI15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EuropeSources" displayName="EuropeSources" ref="A1:AI18" headerRowCount="1">
+  <autoFilter ref="A1:AI18"/>
   <tableColumns count="35">
     <tableColumn id="1" name="Source ID"/>
     <tableColumn id="2" name="Country"/>
@@ -414,8 +414,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="NorthAmericaSources" displayName="NorthAmericaSources" ref="A1:AI5" headerRowCount="1">
-  <autoFilter ref="A1:AI5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="NorthAmericaSources" displayName="NorthAmericaSources" ref="A1:AI8" headerRowCount="1">
+  <autoFilter ref="A1:AI8"/>
   <tableColumns count="35">
     <tableColumn id="1" name="Source ID"/>
     <tableColumn id="2" name="Country"/>
@@ -850,7 +850,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7">
@@ -860,7 +860,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8">
@@ -870,7 +870,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">
@@ -902,7 +902,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -978,7 +978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI9"/>
+  <dimension ref="A1:AI10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -1802,17 +1802,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>kofia_fund_info</t>
+          <t>au_user_managed_funds</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1822,32 +1822,20 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Korea Financial Investment Association</t>
+          <t>User-provided Australian managed-fund dataset</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Fund information one-click system</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>https://fund.kofia.or.kr/fs/fund/html/fundMain.html</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>https://fund.kofia.or.kr/fs/fund/html/fundMain.html</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>https://fund.kofia.or.kr/fs/fund/html/fundMain.html</t>
-        </is>
-      </c>
+          <t>Australian managed-fund metadata catalogue</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Industry association portal</t>
+          <t>User-provided CSV</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1922,56 +1910,46 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>Unavailable</t>
+          <t>Usable Fund Data Confirmed</t>
         </is>
       </c>
       <c r="Z6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>2026-10-17T11:55:49.972662+00:00</t>
-        </is>
-      </c>
+      <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
       <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
-      <c r="AH6" s="2" t="inlineStr">
-        <is>
-          <t>https://fund.kofia.or.kr/fs/fund/html/fundMain.html</t>
-        </is>
-      </c>
+      <c r="AF6" t="n">
+        <v>96</v>
+      </c>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
       <c r="AI6" t="inlineStr">
         <is>
-          <t>KOFIA portal links fund information from regulators, association, managers, and evaluators; source-level provenance and terms must be checked. Capability notes: Fund information; data fields to verify</t>
+          <t>Supplied CSV contains 96 Australian managed-fund records with manager, subcategory, structure, base currency and provider URL. Its ISIN and nav_aud columns are empty for every row, so the import preserves those fields as null. Capability notes: Fund master metadata only; no NAV or ISIN values supplied</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>mas_opera_cis</t>
+          <t>kofia_fund_info</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1981,32 +1959,32 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Monetary Authority of Singapore</t>
+          <t>Korea Financial Investment Association</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>OPERA collective investment scheme register</t>
+          <t>Fund information one-click system</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>https://eservices.mas.gov.sg/opera/Public/CIS/ViewSchemes.aspx</t>
+          <t>https://fund.kofia.or.kr/fs/fund/html/fundMain.html</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>https://eservices.mas.gov.sg/opera/Public/CIS/ViewSchemes.aspx</t>
+          <t>https://fund.kofia.or.kr/fs/fund/html/fundMain.html</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>https://eservices.mas.gov.sg/opera/Public/CIS/ViewSchemes.aspx</t>
+          <t>https://fund.kofia.or.kr/fs/fund/html/fundMain.html</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Government regulator public portal</t>
+          <t>Industry association portal</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -2095,7 +2073,7 @@
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>2026-10-17T11:55:50.026171+00:00</t>
+          <t>2026-10-17T11:55:49.972662+00:00</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr"/>
@@ -2108,29 +2086,29 @@
       </c>
       <c r="AH7" s="2" t="inlineStr">
         <is>
-          <t>https://eservices.mas.gov.sg/opera/Public/CIS/ViewSchemes.aspx</t>
+          <t>https://fund.kofia.or.kr/fs/fund/html/fundMain.html</t>
         </is>
       </c>
       <c r="AI7" t="inlineStr">
         <is>
-          <t>MAS OPERA lists scheme number, name, umbrella, status, and manager, including live examples. It is a register, not a NAV history. Capability notes: Fund master/register fields visible</t>
+          <t>KOFIA portal links fund information from regulators, association, managers, and evaluators; source-level provenance and terms must be checked. Capability notes: Fund information; data fields to verify</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>hk_sfc_authorised_unit_trusts</t>
+          <t>mas_opera_cis</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>HK</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2140,55 +2118,63 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Securities and Futures Commission</t>
+          <t>Monetary Authority of Singapore</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>SFC-authorised unit trusts and mutual funds for public offering</t>
+          <t>OPERA collective investment scheme register</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>https://www.sfc.hk/en/Regulatory-functions/Products/List-of-publicly-offered-investment-products</t>
+          <t>https://eservices.mas.gov.sg/opera/Public/CIS/ViewSchemes.aspx</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>https://apps.sfc.hk/productlistWeb/searchProduct/UTMF.do?lang=EN</t>
+          <t>https://eservices.mas.gov.sg/opera/Public/CIS/ViewSchemes.aspx</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>https://www.sfc.hk/en/Regulatory-functions/Products/List-of-publicly-offered-investment-products</t>
+          <t>https://eservices.mas.gov.sg/opera/Public/CIS/ViewSchemes.aspx</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Government regulator product list</t>
+          <t>Government regulator public portal</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Public SFC product-list HTML; no login</t>
-        </is>
-      </c>
-      <c r="L8" t="b">
-        <v>0</v>
+          <t>Public registry / official website; programmatic access not yet confirmed</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>HTML table; product/sub-fund name, SFC CE number, issuer, authorisation date</t>
-        </is>
-      </c>
-      <c r="N8" t="b">
-        <v>1</v>
-      </c>
-      <c r="O8" t="b">
-        <v>0</v>
-      </c>
-      <c r="P8" t="b">
-        <v>0</v>
+          <t>Unknown — inspect source</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Candidate source</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -2197,22 +2183,22 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>SFC CE number</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Current SFC public-offer product list</t>
+          <t>Not confirmed</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Updated as offering documents are authorised</t>
+          <t>Not confirmed</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -2227,65 +2213,61 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>Unknown — confirm SFC reuse terms</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>Usable Fund Data Confirmed</t>
+          <t>Unavailable</t>
         </is>
       </c>
       <c r="Z8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>Integrated</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>2026-10-18T19:45:12.781623+00:00</t>
-        </is>
-      </c>
-      <c r="AD8" t="inlineStr">
-        <is>
-          <t>2026-10-18T19:45:12.781623+00:00</t>
-        </is>
-      </c>
-      <c r="AE8" t="n">
-        <v>2255</v>
-      </c>
-      <c r="AF8" t="n">
-        <v>2255</v>
-      </c>
-      <c r="AG8" t="inlineStr"/>
+          <t>2026-10-17T11:55:50.026171+00:00</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
       <c r="AH8" s="2" t="inlineStr">
         <is>
-          <t>https://www.sfc.hk/en/Regulatory-functions/Products/List-of-publicly-offered-investment-products</t>
+          <t>https://eservices.mas.gov.sg/opera/Public/CIS/ViewSchemes.aspx</t>
         </is>
       </c>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>Records are products authorized for public offering in Hong Kong, not necessarily domiciled there. Domicile, currency and NAV are left null; this source is market-availability coverage.</t>
+          <t>MAS OPERA lists scheme number, name, umbrella, status, and manager, including live examples. It is a register, not a NAV history. Capability notes: Fund master/register fields visible</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>sitca_fund_info</t>
+          <t>hk_sfc_authorised_unit_trusts</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Taiwan</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>HK</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2295,37 +2277,37 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Securities and Futures Bureau / SITCA</t>
+          <t>Securities and Futures Commission</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Daily NAV of Domestic Funds</t>
+          <t>SFC-authorised unit trusts and mutual funds for public offering</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.tw/en/datasets/11109</t>
+          <t>https://www.sfc.hk/en/Regulatory-functions/Products/List-of-publicly-offered-investment-products</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>https://www.sitca.org.tw/MemberK0000/F/03/nav.csv</t>
+          <t>https://apps.sfc.hk/productlistWeb/searchProduct/UTMF.do?lang=EN</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.tw/en/datasets/11109</t>
+          <t>https://www.sfc.hk/en/Regulatory-functions/Products/List-of-publicly-offered-investment-products</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Government open-data CSV</t>
+          <t>Government regulator product list</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Public CSV listed by Taiwan government open-data catalog</t>
+          <t>Public SFC product-list HTML; no login</t>
         </is>
       </c>
       <c r="L9" t="b">
@@ -2333,101 +2315,246 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>CSV</t>
+          <t>HTML table; product/sub-fund name, SFC CE number, issuer, authorisation date</t>
         </is>
       </c>
       <c r="N9" t="b">
         <v>1</v>
       </c>
       <c r="O9" t="b">
+        <v>0</v>
+      </c>
+      <c r="P9" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>SFC CE number</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Current SFC public-offer product list</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Updated as offering documents are authorised</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Unknown — confirm SFC reuse terms</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>Usable Fund Data Confirmed</t>
+        </is>
+      </c>
+      <c r="Z9" t="b">
         <v>1</v>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>Current daily file; archive bounds to verify</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>Currency</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>Fund code, beneficiary certificate code, tax ID</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>To verify from downloadable resource</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Daily</t>
-        </is>
-      </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>Not confirmed</t>
-        </is>
-      </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>Permitted</t>
-        </is>
-      </c>
-      <c r="X9" t="inlineStr">
-        <is>
-          <t>Permitted under Open Government Data License 1.0; confirm attribution terms</t>
-        </is>
-      </c>
-      <c r="Y9" t="inlineStr">
-        <is>
-          <t>Unavailable</t>
-        </is>
-      </c>
-      <c r="Z9" t="b">
-        <v>0</v>
-      </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>2026-10-17T11:55:50.133422+00:00</t>
-        </is>
-      </c>
+      <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr"/>
       <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr"/>
-      <c r="AG9" t="inlineStr">
+      <c r="AF9" t="n">
+        <v>2255</v>
+      </c>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sfc.hk/en/Regulatory-functions/Products/List-of-publicly-offered-investment-products</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>Records are products authorized for public offering in Hong Kong, not necessarily domiciled there. Domicile, currency and NAV are left null; this source is market-availability coverage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>sitca_fund_info</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Asia-Pacific</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Securities and Futures Bureau / SITCA</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Daily NAV of Domestic Funds</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>https://data.gov.tw/en/datasets/11109</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sitca.org.tw/MemberK0000/F/03/nav.csv</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>https://data.gov.tw/en/datasets/11109</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Government open-data CSV</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Public CSV listed by Taiwan government open-data catalog</t>
+        </is>
+      </c>
+      <c r="L10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="N10" t="b">
+        <v>1</v>
+      </c>
+      <c r="O10" t="b">
+        <v>1</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Current daily file; archive bounds to verify</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Fund code, beneficiary certificate code, tax ID</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>To verify from downloadable resource</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Permitted</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>Permitted under Open Government Data License 1.0; confirm attribution terms</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>Unavailable</t>
+        </is>
+      </c>
+      <c r="Z10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:55:50.133422+00:00</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr">
         <is>
           <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
         </is>
       </c>
-      <c r="AH9" s="2" t="inlineStr">
+      <c r="AH10" s="2" t="inlineStr">
         <is>
           <t>https://data.gov.tw/en/datasets/11109</t>
         </is>
       </c>
-      <c r="AI9" t="inlineStr">
+      <c r="AI10" t="inlineStr">
         <is>
           <t>Government catalog confirms daily fund-level NAV fields, free access and Open Government Data License 1.0. Publisher CSV timed out from this runtime; no download or ingestion has succeeded yet.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AI9"/>
-  <conditionalFormatting sqref="Y2:Y9">
+  <autoFilter ref="A1:AI10"/>
+  <conditionalFormatting sqref="Y2:Y10">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>OR(Y2="Usable Fund Data Confirmed",Y2="Reachable")</formula>
     </cfRule>
@@ -2435,7 +2562,7 @@
       <formula>OR(Y2="Blocked",Y2="Unavailable")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA2:AA9">
+  <conditionalFormatting sqref="AA2:AA10">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AA2="Integrated"</formula>
     </cfRule>
@@ -2444,13 +2571,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="W2:W9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="W2:W10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Permitted,Restricted,Permission Required,Unknown"</formula1>
     </dataValidation>
-    <dataValidation sqref="Y2:Y9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Y2:Y10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Undiscovered,Discovered,Reachable,Authentication Required,Blocked,Unavailable,Accessible — No Fund Data,Usable Fund Data Confirmed"</formula1>
     </dataValidation>
-    <dataValidation sqref="AA2:AA9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AA2:AA10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,In Progress,Implemented,Tested,Integrated,Failed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2471,22 +2598,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH5" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH6" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH7" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH8" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH9" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH7" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH8" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH9" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH10" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -2501,10 +2628,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI15"/>
+  <dimension ref="A1:AI18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -3305,7 +3432,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>fca_authorised_funds</t>
+          <t>uk_fundslibrary_unit_prices</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3325,55 +3452,63 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Financial Conduct Authority</t>
+          <t>FundsLibrary</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>UK authorised and recognised fund register</t>
+          <t>UK public unit-price table</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>https://www.fca.org.uk/freedom-information/information-consumer-investment-june-2026</t>
+          <t>https://www.fundslibrary.co.uk/FundsLibrary.BrandedTools/OnlineIps/FundCentral/Collective/UnitPrices</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>https://www.fca.org.uk/publication/fca/foi2026_01166-annex-a.csv</t>
+          <t>https://www.fundslibrary.co.uk/FundsLibrary.BrandedTools/OnlineIps/FundCentral/Collective/UnitPrices</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>https://www.fca.org.uk/freedom-information/information-consumer-investment-june-2026</t>
+          <t>https://www.fundslibrary.co.uk/FundsLibrary.BrandedTools/OnlineIps/FundCentral/Collective/UnitPrices</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Government regulator CSV snapshot</t>
+          <t>Public fund platform table</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Public FCA CSV download; no login</t>
-        </is>
-      </c>
-      <c r="L6" t="b">
-        <v>0</v>
+          <t>Public registry / official website; programmatic access not yet confirmed</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>CSV; Windows-1252; 11,842 product rows in the 2026-06 snapshot</t>
-        </is>
-      </c>
-      <c r="N6" t="b">
-        <v>1</v>
-      </c>
-      <c r="O6" t="b">
-        <v>0</v>
-      </c>
-      <c r="P6" t="b">
-        <v>0</v>
+          <t>Unknown — inspect source</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Candidate source</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -3382,22 +3517,22 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>FCA Product Reference Number (PRN)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Snapshot published 2026-06-24</t>
+          <t>Not confirmed</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Snapshot publication; refresh when FCA posts a new file</t>
+          <t>Not confirmed</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -3412,7 +3547,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>Unknown — confirm FCA reuse terms</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -3433,34 +3568,34 @@
       <c r="AD6" t="inlineStr"/>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="n">
-        <v>3975</v>
+        <v>33</v>
       </c>
       <c r="AG6" t="inlineStr"/>
       <c r="AH6" s="2" t="inlineStr">
         <is>
-          <t>https://www.fca.org.uk/freedom-information/information-consumer-investment-june-2026</t>
+          <t>https://www.fundslibrary.co.uk/FundsLibrary.BrandedTools/OnlineIps/FundCentral/Collective/UnitPrices</t>
         </is>
       </c>
       <c r="AI6" t="inlineStr">
         <is>
-          <t>Imported rows are limited to FCA statuses Authorised and Approved, which FCA identifies as UK-domiciled. Recognised offshore rows are excluded. Currency and NAV remain null/not loaded.</t>
+          <t>Public table provides fund name, SEDOL, Investment Association sector, status, price date and NAV price in pence. This snapshot yielded 33 usable rows; it is an issuer/platform catalogue, not the complete FCA-authorised universe. Capability notes: 33 UK fund NAV observations with IA sectors</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>de_bde_nonmonetary_funds</t>
+          <t>uk_ft_morningstar_prices</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -3470,55 +3605,63 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Banco de España</t>
+          <t>Financial Times / ICE Data Services</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>List of non-monetary investment funds in Germany</t>
+          <t>Public UK fund price table (Morningstar/FT archive)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-de.html</t>
+          <t>https://markets.ft.markitdigital.com/data/dataarchive/ajax/fetchreport?documentKey=688_UTS~Combined_261024&amp;reportCode=UTS_Combined</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-de.csv</t>
+          <t>https://markets.ft.markitdigital.com/data/dataarchive/ajax/fetchreport?documentKey=688_UTS~Combined_261024&amp;reportCode=UTS_Combined</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-de.html</t>
+          <t>https://markets.ft.markitdigital.com/data/dataarchive/ajax/fetchreport?documentKey=688_UTS~Combined_261024&amp;reportCode=UTS_Combined</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Official statistical fund register CSV</t>
+          <t>Public market-data archive</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Public Banco de España country-level CSV; no login</t>
-        </is>
-      </c>
-      <c r="L7" t="b">
-        <v>0</v>
+          <t>Public registry / official website; programmatic access not yet confirmed</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>UTF-8 CSV; fund code, LEI, name, manager, address, policy and open/closed status</t>
-        </is>
-      </c>
-      <c r="N7" t="b">
-        <v>1</v>
-      </c>
-      <c r="O7" t="b">
-        <v>0</v>
-      </c>
-      <c r="P7" t="b">
-        <v>0</v>
+          <t>Unknown — inspect source</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Candidate source</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -3527,22 +3670,22 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>European code; LEI where present</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Current fund-register snapshot</t>
+          <t>Not confirmed</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Snapshot; check for updates</t>
+          <t>Not confirmed</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -3557,7 +3700,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>Unknown — confirm Banco de España reuse terms</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
@@ -3578,34 +3721,34 @@
       <c r="AD7" t="inlineStr"/>
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="n">
-        <v>6400</v>
+        <v>253</v>
       </c>
       <c r="AG7" t="inlineStr"/>
       <c r="AH7" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-de.html</t>
+          <t>https://markets.ft.markitdigital.com/data/dataarchive/ajax/fetchreport?documentKey=688_UTS~Combined_261024&amp;reportCode=UTS_Combined</t>
         </is>
       </c>
       <c r="AI7" t="inlineStr">
         <is>
-          <t>Imports only open-ended non-monetary investment fund entries for this domicile. Register includes UCITS and AIF categories; it is broader than a strict UCITS-only universe. No NAV or currency is inferred.</t>
+          <t>Public FT archive table of manager-supplied bid prices, collated by ICE and sourced from Morningstar/FT fund data. Prices are in pence unless a currency symbol is shown; this snapshot yielded 253 rows. Bid price is a quoted fund price and is not asserted to be an official regulator NAV. Capability notes: 253 UK fund price observations; no ISIN in this table</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>amf_geco</t>
+          <t>de_bundesanzeiger_navs</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -3615,55 +3758,63 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Autorité des marchés financiers</t>
+          <t>Bundesanzeiger / Federal Gazette</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>GECO French-domiciled OPC product/share-class export</t>
+          <t>Public German-market fund prices and NAVs (Fondsdata)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>https://geco.amf-france.org/liste-des-produits-d-epargne</t>
+          <t>https://www.bundesanzeiger.de/pub/en/fondsdata</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>https://geco.amf-france.org/back-office/funds/compartments</t>
+          <t>https://www.bundesanzeiger.de/pub/en/fondsdata</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>https://geco.amf-france.org/liste-des-produits-d-epargne</t>
+          <t>https://www.bundesanzeiger.de/pub/en/fondsdata</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Government regulator JSON export</t>
+          <t>Government publication platform</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Public AMF GECO JSON export using the web client request format</t>
-        </is>
-      </c>
-      <c r="L8" t="b">
-        <v>0</v>
+          <t>Public registry / official website; programmatic access not yet confirmed</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>JSON; product and compartment/share-class records</t>
-        </is>
-      </c>
-      <c r="N8" t="b">
-        <v>1</v>
-      </c>
-      <c r="O8" t="b">
-        <v>0</v>
-      </c>
-      <c r="P8" t="b">
-        <v>0</v>
+          <t>Unknown — inspect source</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Candidate source</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -3672,22 +3823,22 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>None in this export</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>AMF compartment ID, AMF product ID and ISIN where present</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Current active product snapshot; no NAV history</t>
+          <t>Not confirmed</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Current export on demand</t>
+          <t>Not confirmed</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -3702,63 +3853,64 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>Unknown — confirm AMF reuse terms</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>Usable Fund Data Confirmed</t>
+          <t>Discovered</t>
         </is>
       </c>
       <c r="Z8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>Integrated</t>
+          <t>Failed</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="inlineStr">
-        <is>
-          <t>2026-10-17T11:55:49.437058+00:00</t>
-        </is>
-      </c>
+      <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="inlineStr"/>
+      <c r="AE8" t="n">
+        <v>249</v>
+      </c>
       <c r="AF8" t="n">
-        <v>28375</v>
+        <v>127</v>
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+          <t>ValidationError: 1 validation error for CanonicalNav
+nav
+  Input should be greater than 0 [type=greater_than, input_value='0.0', input_type=str]
+    For further information visit https://errors.pydantic.dev/2.14/v/greater_than</t>
         </is>
       </c>
       <c r="AH8" s="2" t="inlineStr">
         <is>
-          <t>https://geco.amf-france.org/liste-des-produits-d-epargne</t>
+          <t>https://www.bundesanzeiger.de/pub/en/fondsdata</t>
         </is>
       </c>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>ETL filters active French-domiciled products and expands available share-class ISINs. Foreign-domiciled products authorised for marketing in France are excluded. No currency or NAV is inferred.</t>
+          <t>Fondsdata publishes fund name, provider, ISIN/WKN, date, offer price, bid price, currency and NAV. This import collected 249 unique public rows from paginated free search results; dates are the latest result returned per ISIN and can differ by fund. German domicile is set only for DE-prefixed ISINs; other rows are foreign funds published in the German market. Capability notes: 249 fund/share-class NAV observations with ISIN and currency</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>finma_swiss_fund_list</t>
+          <t>fca_authorised_funds</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -3768,37 +3920,37 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Swiss Financial Market Supervisory Authority</t>
+          <t>Financial Conduct Authority</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Approved Swiss collective investment schemes</t>
+          <t>UK authorised and recognised fund register</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>https://www.finma.ch/en/finma-public/authorised-institutions-individuals-and-products/</t>
+          <t>https://www.fca.org.uk/freedom-information/information-consumer-investment-june-2026</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>https://www.finma.ch/~/media/finma/dokumente/bewilligungstraeger/pdf/afch.pdf?la=en%3BApproved</t>
+          <t>https://www.fca.org.uk/publication/fca/foi2026_01166-annex-a.csv</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>https://www.finma.ch/en/finma-public/authorised-institutions-individuals-and-products/</t>
+          <t>https://www.fca.org.uk/freedom-information/information-consumer-investment-june-2026</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Government regulator PDF</t>
+          <t>Government regulator CSV snapshot</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Public FINMA PDF download; no login</t>
+          <t>Public FCA CSV download; no login</t>
         </is>
       </c>
       <c r="L9" t="b">
@@ -3806,7 +3958,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>PDF; tabular list with individual fund name and FINMA-ID</t>
+          <t>CSV; Windows-1252; 11,842 product rows in the 2026-06 snapshot</t>
         </is>
       </c>
       <c r="N9" t="b">
@@ -3825,22 +3977,22 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>None in approved-funds list</t>
+          <t>None</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>FINMA-ID</t>
+          <t>FCA Product Reference Number (PRN)</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Current approved-funds list, dated 2026-10-18</t>
+          <t>Snapshot published 2026-06-24</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>FINMA republishes the register periodically</t>
+          <t>Snapshot publication; refresh when FCA posts a new file</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -3855,7 +4007,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>Unknown — confirm FINMA reuse terms</t>
+          <t>Unknown — confirm FCA reuse terms</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
@@ -3876,34 +4028,34 @@
       <c r="AD9" t="inlineStr"/>
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="n">
-        <v>2007</v>
+        <v>3975</v>
       </c>
       <c r="AG9" t="inlineStr"/>
       <c r="AH9" s="2" t="inlineStr">
         <is>
-          <t>https://www.finma.ch/en/finma-public/authorised-institutions-individuals-and-products/</t>
+          <t>https://www.fca.org.uk/freedom-information/information-consumer-investment-june-2026</t>
         </is>
       </c>
       <c r="AI9" t="inlineStr">
         <is>
-          <t>The FINMA domestic approved-schemes PDF has individual fund/sub-fund names and FINMA IDs. The connector imports those product rows; it does not infer currency or NAV.</t>
+          <t>Imported rows are limited to FCA statuses Authorised and Approved, which FCA identifies as UK-domiciled. Recognised offshore rows are excluded. Currency and NAV remain null/not loaded.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>nl_bde_nonmonetary_funds</t>
+          <t>de_bde_nonmonetary_funds</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>NL</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -3918,22 +4070,22 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>List of non-monetary investment funds in the Netherlands</t>
+          <t>List of non-monetary investment funds in Germany</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-nl.html</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-de.html</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-nl.csv</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-de.csv</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-nl.html</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-de.html</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -4021,12 +4173,12 @@
       <c r="AD10" t="inlineStr"/>
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="n">
-        <v>1306</v>
+        <v>6400</v>
       </c>
       <c r="AG10" t="inlineStr"/>
       <c r="AH10" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-nl.html</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-de.html</t>
         </is>
       </c>
       <c r="AI10" t="inlineStr">
@@ -4038,17 +4190,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>dk_bde_nonmonetary_funds</t>
+          <t>amf_geco</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>DK</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -4058,37 +4210,37 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Banco de España</t>
+          <t>Autorité des marchés financiers</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>List of non-monetary investment funds in Denmark</t>
+          <t>GECO French-domiciled OPC product/share-class export</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-dk.html</t>
+          <t>https://geco.amf-france.org/liste-des-produits-d-epargne</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-dk.csv</t>
+          <t>https://geco.amf-france.org/back-office/funds/compartments</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-dk.html</t>
+          <t>https://geco.amf-france.org/liste-des-produits-d-epargne</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Official national statistical register CSV</t>
+          <t>Government regulator JSON export</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Public CSV download; no login</t>
+          <t>Public AMF GECO JSON export using the web client request format</t>
         </is>
       </c>
       <c r="L11" t="b">
@@ -4096,7 +4248,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>CSV; UTF-8; seven published columns plus an empty padded column</t>
+          <t>JSON; product and compartment/share-class records</t>
         </is>
       </c>
       <c r="N11" t="b">
@@ -4115,22 +4267,22 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None in this export</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>European code, LEI where present</t>
+          <t>AMF compartment ID, AMF product ID and ISIN where present</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Current register snapshot</t>
+          <t>Current active product snapshot; no NAV history</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Register snapshot; check source for updates</t>
+          <t>Current export on demand</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -4145,7 +4297,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>Unknown — confirm Banco de España reuse terms</t>
+          <t>Unknown — confirm AMF reuse terms</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
@@ -4162,38 +4314,46 @@
         </is>
       </c>
       <c r="AB11" t="inlineStr"/>
-      <c r="AC11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:55:49.437058+00:00</t>
+        </is>
+      </c>
       <c r="AD11" t="inlineStr"/>
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="n">
-        <v>1486</v>
-      </c>
-      <c r="AG11" t="inlineStr"/>
+        <v>28375</v>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
       <c r="AH11" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-dk.html</t>
+          <t>https://geco.amf-france.org/liste-des-produits-d-epargne</t>
         </is>
       </c>
       <c r="AI11" t="inlineStr">
         <is>
-          <t>Imports open-ended Danish non-monetary investment funds only. The source also includes AIFs, so this is broader than a strict UCITS mutual-fund universe. No currency or NAV is inferred.</t>
+          <t>ETL filters active French-domiciled products and expands available share-class ISINs. Foreign-domiciled products authorised for marketing in France are excluded. No currency or NAV is inferred.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>fi_fund_holdings</t>
+          <t>finma_swiss_fund_list</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -4203,63 +4363,55 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Finansinspektionen</t>
+          <t>Swiss Financial Market Supervisory Authority</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Fund holdings register</t>
+          <t>Approved Swiss collective investment schemes</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>https://www.fi.se/en/our-registers/fund-holdings/</t>
+          <t>https://www.finma.ch/en/finma-public/authorised-institutions-individuals-and-products/</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>https://www.fi.se/en/our-registers/fund-holdings/</t>
+          <t>https://www.finma.ch/~/media/finma/dokumente/bewilligungstraeger/pdf/afch.pdf?la=en%3BApproved</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>https://www.fi.se/en/our-registers/fund-holdings/</t>
+          <t>https://www.finma.ch/en/finma-public/authorised-institutions-individuals-and-products/</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Government regulator reporting data</t>
+          <t>Government regulator PDF</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Public registry / official website; programmatic access not yet confirmed</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
+          <t>Public FINMA PDF download; no login</t>
+        </is>
+      </c>
+      <c r="L12" t="b">
+        <v>0</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Unknown — inspect source</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>Candidate source</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
+          <t>PDF; tabular list with individual fund name and FINMA-ID</t>
+        </is>
+      </c>
+      <c r="N12" t="b">
+        <v>1</v>
+      </c>
+      <c r="O12" t="b">
+        <v>0</v>
+      </c>
+      <c r="P12" t="b">
+        <v>0</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -4268,29 +4420,29 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>None in approved-funds list</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>FINMA-ID</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
+          <t>Current approved-funds list, dated 2026-10-18</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>FINMA republishes the register periodically</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
           <t>Not confirmed</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>Not confirmed</t>
-        </is>
-      </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>Not confirmed</t>
-        </is>
-      </c>
       <c r="W12" t="inlineStr">
         <is>
           <t>Unknown</t>
@@ -4298,61 +4450,55 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Unknown — confirm FINMA reuse terms</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>Unavailable</t>
+          <t>Usable Fund Data Confirmed</t>
         </is>
       </c>
       <c r="Z12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr"/>
-      <c r="AC12" t="inlineStr">
-        <is>
-          <t>2026-10-17T11:55:49.651051+00:00</t>
-        </is>
-      </c>
+      <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="inlineStr"/>
       <c r="AE12" t="inlineStr"/>
-      <c r="AF12" t="inlineStr"/>
-      <c r="AG12" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+      <c r="AF12" t="n">
+        <v>2007</v>
+      </c>
+      <c r="AG12" t="inlineStr"/>
       <c r="AH12" s="2" t="inlineStr">
         <is>
-          <t>https://www.fi.se/en/our-registers/fund-holdings/</t>
+          <t>https://www.finma.ch/en/finma-public/authorised-institutions-individuals-and-products/</t>
         </is>
       </c>
       <c r="AI12" t="inlineStr">
         <is>
-          <t>FI publishes fund holdings data; special-fund holdings are excluded. This supports holdings research, not fund NAV coverage. Capability notes: Fund holdings; NAV not confirmed</t>
+          <t>The FINMA domestic approved-schemes PDF has individual fund/sub-fund names and FINMA IDs. The connector imports those product rows; it does not infer currency or NAV.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>lu_bde_nonmonetary_funds</t>
+          <t>nl_bde_nonmonetary_funds</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>LU</t>
+          <t>NL</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -4367,22 +4513,22 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>List of non-monetary investment funds in Luxembourg</t>
+          <t>List of non-monetary investment funds in the Netherlands</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-lu.html</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-nl.html</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-lu.csv</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-nl.csv</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-lu.html</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-nl.html</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -4470,12 +4616,12 @@
       <c r="AD13" t="inlineStr"/>
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="n">
-        <v>23955</v>
+        <v>1306</v>
       </c>
       <c r="AG13" t="inlineStr"/>
       <c r="AH13" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-lu.html</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-nl.html</t>
         </is>
       </c>
       <c r="AI13" t="inlineStr">
@@ -4487,17 +4633,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>cbI_fund_registers</t>
+          <t>dk_bde_nonmonetary_funds</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>IE</t>
+          <t>DK</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -4507,63 +4653,55 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Central Bank of Ireland</t>
+          <t>Banco de España</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Collective investment scheme registers and downloads</t>
+          <t>List of non-monetary investment funds in Denmark</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>https://registers.centralbank.ie/downloadspage.aspx</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-dk.html</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>https://registers.centralbank.ie/downloadspage.aspx</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-dk.csv</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>https://registers.centralbank.ie/downloadspage.aspx</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-dk.html</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Government regulator register and downloads</t>
+          <t>Official national statistical register CSV</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Public registry / official website; programmatic access not yet confirmed</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
+          <t>Public CSV download; no login</t>
+        </is>
+      </c>
+      <c r="L14" t="b">
+        <v>0</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Unknown — inspect source</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>Candidate source</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
+          <t>CSV; UTF-8; seven published columns plus an empty padded column</t>
+        </is>
+      </c>
+      <c r="N14" t="b">
+        <v>1</v>
+      </c>
+      <c r="O14" t="b">
+        <v>0</v>
+      </c>
+      <c r="P14" t="b">
+        <v>0</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -4572,29 +4710,29 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>None</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>European code, LEI where present</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
+          <t>Current register snapshot</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Register snapshot; check source for updates</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
           <t>Not confirmed</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>Not confirmed</t>
-        </is>
-      </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>Not confirmed</t>
-        </is>
-      </c>
       <c r="W14" t="inlineStr">
         <is>
           <t>Unknown</t>
@@ -4602,61 +4740,55 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Unknown — confirm Banco de España reuse terms</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>Unavailable</t>
+          <t>Usable Fund Data Confirmed</t>
         </is>
       </c>
       <c r="Z14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="AB14" t="inlineStr"/>
-      <c r="AC14" t="inlineStr">
-        <is>
-          <t>2026-10-17T11:55:49.758179+00:00</t>
-        </is>
-      </c>
+      <c r="AC14" t="inlineStr"/>
       <c r="AD14" t="inlineStr"/>
       <c r="AE14" t="inlineStr"/>
-      <c r="AF14" t="inlineStr"/>
-      <c r="AG14" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+      <c r="AF14" t="n">
+        <v>1486</v>
+      </c>
+      <c r="AG14" t="inlineStr"/>
       <c r="AH14" s="2" t="inlineStr">
         <is>
-          <t>https://registers.centralbank.ie/downloadspage.aspx</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-dk.html</t>
         </is>
       </c>
       <c r="AI14" t="inlineStr">
         <is>
-          <t>Official CIS search and downloads include authorised funds and UCITS lists, generally PDF; monthly fund-data publications are available, format suitability needs inspection. Capability notes: Fund master; monthly fund reports</t>
+          <t>Imports open-ended Danish non-monetary investment funds only. The source also includes AIFs, so this is broader than a strict UCITS mutual-fund universe. No currency or NAV is inferred.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>it_bde_nonmonetary_funds</t>
+          <t>fi_fund_holdings</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -4666,55 +4798,63 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Banco de España</t>
+          <t>Finansinspektionen</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>List of non-monetary investment funds in Italy</t>
+          <t>Fund holdings register</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-it.html</t>
+          <t>https://www.fi.se/en/our-registers/fund-holdings/</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-it.csv</t>
+          <t>https://www.fi.se/en/our-registers/fund-holdings/</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-it.html</t>
+          <t>https://www.fi.se/en/our-registers/fund-holdings/</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Official statistical fund register CSV</t>
+          <t>Government regulator reporting data</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Public Banco de España country-level CSV; no login</t>
-        </is>
-      </c>
-      <c r="L15" t="b">
-        <v>0</v>
+          <t>Public registry / official website; programmatic access not yet confirmed</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>UTF-8 CSV; fund code, LEI, name, manager, address, policy and open/closed status</t>
-        </is>
-      </c>
-      <c r="N15" t="b">
-        <v>1</v>
-      </c>
-      <c r="O15" t="b">
-        <v>0</v>
-      </c>
-      <c r="P15" t="b">
-        <v>0</v>
+          <t>Unknown — inspect source</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Candidate source</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -4723,22 +4863,22 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>European code; LEI where present</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Current fund-register snapshot</t>
+          <t>Not confirmed</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Snapshot; check for updates</t>
+          <t>Not confirmed</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
@@ -4753,44 +4893,499 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>Unknown — confirm Banco de España reuse terms</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>Usable Fund Data Confirmed</t>
+          <t>Unavailable</t>
         </is>
       </c>
       <c r="Z15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>Integrated</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr"/>
-      <c r="AC15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:55:49.651051+00:00</t>
+        </is>
+      </c>
       <c r="AD15" t="inlineStr"/>
       <c r="AE15" t="inlineStr"/>
-      <c r="AF15" t="n">
+      <c r="AF15" t="inlineStr"/>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
+      <c r="AH15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fi.se/en/our-registers/fund-holdings/</t>
+        </is>
+      </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>FI publishes fund holdings data; special-fund holdings are excluded. This supports holdings research, not fund NAV coverage. Capability notes: Fund holdings; NAV not confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>lu_bde_nonmonetary_funds</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Luxembourg</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>LU</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Banco de España</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>List of non-monetary investment funds in Luxembourg</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-lu.html</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-lu.csv</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-lu.html</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Official statistical fund register CSV</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Public Banco de España country-level CSV; no login</t>
+        </is>
+      </c>
+      <c r="L16" t="b">
+        <v>0</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>UTF-8 CSV; fund code, LEI, name, manager, address, policy and open/closed status</t>
+        </is>
+      </c>
+      <c r="N16" t="b">
+        <v>1</v>
+      </c>
+      <c r="O16" t="b">
+        <v>0</v>
+      </c>
+      <c r="P16" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>European code; LEI where present</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Current fund-register snapshot</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Snapshot; check for updates</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>Unknown — confirm Banco de España reuse terms</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>Usable Fund Data Confirmed</t>
+        </is>
+      </c>
+      <c r="Z16" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>Integrated</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
+      <c r="AD16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="n">
+        <v>23955</v>
+      </c>
+      <c r="AG16" t="inlineStr"/>
+      <c r="AH16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-lu.html</t>
+        </is>
+      </c>
+      <c r="AI16" t="inlineStr">
+        <is>
+          <t>Imports only open-ended non-monetary investment fund entries for this domicile. Register includes UCITS and AIF categories; it is broader than a strict UCITS-only universe. No NAV or currency is inferred.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>cbI_fund_registers</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>IE</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Central Bank of Ireland</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Collective investment scheme registers and downloads</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>https://registers.centralbank.ie/downloadspage.aspx</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>https://registers.centralbank.ie/downloadspage.aspx</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>https://registers.centralbank.ie/downloadspage.aspx</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Government regulator register and downloads</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Public registry / official website; programmatic access not yet confirmed</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Unknown — inspect source</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Candidate source</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>Unavailable</t>
+        </is>
+      </c>
+      <c r="Z17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:55:49.758179+00:00</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr"/>
+      <c r="AE17" t="inlineStr"/>
+      <c r="AF17" t="inlineStr"/>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
+      <c r="AH17" s="2" t="inlineStr">
+        <is>
+          <t>https://registers.centralbank.ie/downloadspage.aspx</t>
+        </is>
+      </c>
+      <c r="AI17" t="inlineStr">
+        <is>
+          <t>Official CIS search and downloads include authorised funds and UCITS lists, generally PDF; monthly fund-data publications are available, format suitability needs inspection. Capability notes: Fund master; monthly fund reports</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>it_bde_nonmonetary_funds</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Banco de España</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>List of non-monetary investment funds in Italy</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-it.html</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-it.csv</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-it.html</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Official statistical fund register CSV</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Public Banco de España country-level CSV; no login</t>
+        </is>
+      </c>
+      <c r="L18" t="b">
+        <v>0</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>UTF-8 CSV; fund code, LEI, name, manager, address, policy and open/closed status</t>
+        </is>
+      </c>
+      <c r="N18" t="b">
+        <v>1</v>
+      </c>
+      <c r="O18" t="b">
+        <v>0</v>
+      </c>
+      <c r="P18" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>European code; LEI where present</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Current fund-register snapshot</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Snapshot; check for updates</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>Unknown — confirm Banco de España reuse terms</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>Usable Fund Data Confirmed</t>
+        </is>
+      </c>
+      <c r="Z18" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>Integrated</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
+      <c r="AD18" t="inlineStr"/>
+      <c r="AE18" t="inlineStr"/>
+      <c r="AF18" t="n">
         <v>1326</v>
       </c>
-      <c r="AG15" t="inlineStr"/>
-      <c r="AH15" s="2" t="inlineStr">
+      <c r="AG18" t="inlineStr"/>
+      <c r="AH18" s="2" t="inlineStr">
         <is>
           <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-it.html</t>
         </is>
       </c>
-      <c r="AI15" t="inlineStr">
+      <c r="AI18" t="inlineStr">
         <is>
           <t>Imports only open-ended non-monetary investment fund entries for this domicile. Register includes UCITS and AIF categories; it is broader than a strict UCITS-only universe. No NAV or currency is inferred.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AI15"/>
-  <conditionalFormatting sqref="Y2:Y15">
+  <autoFilter ref="A1:AI18"/>
+  <conditionalFormatting sqref="Y2:Y18">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>OR(Y2="Usable Fund Data Confirmed",Y2="Reachable")</formula>
     </cfRule>
@@ -4798,7 +5393,7 @@
       <formula>OR(Y2="Blocked",Y2="Unavailable")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA2:AA15">
+  <conditionalFormatting sqref="AA2:AA18">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AA2="Integrated"</formula>
     </cfRule>
@@ -4807,13 +5402,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="W2:W15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="W2:W18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Permitted,Restricted,Permission Required,Unknown"</formula1>
     </dataValidation>
-    <dataValidation sqref="Y2:Y15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Y2:Y18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Undiscovered,Discovered,Reachable,Authentication Required,Blocked,Unavailable,Accessible — No Fund Data,Usable Fund Data Confirmed"</formula1>
     </dataValidation>
-    <dataValidation sqref="AA2:AA15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AA2:AA18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,In Progress,Implemented,Tested,Integrated,Failed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4874,10 +5469,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH15" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH16" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH17" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH18" r:id="rId68"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId57"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId69"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4888,7 +5495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI5"/>
+  <dimension ref="A1:AI8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5543,17 +6150,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>cnbv_fund_statistics</t>
+          <t>us_qqqm_etf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -5563,32 +6170,32 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Comisión Nacional Bancaria y de Valores</t>
+          <t>Invesco</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Investment fund statistical information</t>
+          <t>Invesco NASDAQ 100 ETF (QQQM)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>https://www.gob.mx/cnbv/acciones-y-programas/informacion-estadistica-fondos-de-inversion</t>
+          <t>https://www.invesco.com/us/en/financial-products/etfs/invesco-nasdaq-100-etf.html</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>https://www.gob.mx/cnbv/acciones-y-programas/informacion-estadistica-fondos-de-inversion</t>
+          <t>https://www.invesco.com/us/en/financial-products/etfs/invesco-nasdaq-100-etf.html</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>https://www.gob.mx/cnbv/acciones-y-programas/informacion-estadistica-fondos-de-inversion</t>
+          <t>https://www.invesco.com/us/en/financial-products/etfs/invesco-nasdaq-100-etf.html</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Government regulator; statistical portal</t>
+          <t>Asset manager page plus public price endpoint</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -5663,45 +6270,504 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>Unavailable</t>
+          <t>Usable Fund Data Confirmed</t>
         </is>
       </c>
       <c r="Z5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>2026-10-17T11:55:49.331740+00:00</t>
-        </is>
-      </c>
+      <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr"/>
       <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr">
+      <c r="AF5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.invesco.com/us/en/financial-products/etfs/invesco-nasdaq-100-etf.html</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>Verified ETF identity: ticker QQQM, ISIN US46138G6492, CUSIP 46138G649, USD. Daily NAV/close is loaded separately from a public Yahoo chart response; Morningstar reference page is retained as research context. Capability notes: Single ETF identity and daily NAV</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>scotia_canada_daily_nav</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Scotiabank / ScotiaFunds</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Daily Canadian mutual-fund NAV workbook</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.scotiafunds.com/en/home/all-funds/mutual-fund</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.scotiafunds.com/en/home/all-funds/mutual-fund</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.scotiafunds.com/en/home/all-funds/mutual-fund</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Fund manager XLSX</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Public registry / official website; programmatic access not yet confirmed</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Unknown — inspect source</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Candidate source</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Usable Fund Data Confirmed</t>
+        </is>
+      </c>
+      <c r="Z6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>Integrated</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="n">
+        <v>373</v>
+      </c>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.scotiafunds.com/en/home/all-funds/mutual-fund</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>Official Scotia workbook contains fund name, series, fund code, currency, valuation date and daily NAV. Broad category is derived from fund-name keywords because the workbook does not publish a category column. Capability notes: 373 Canadian fund/share-class NAV rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>bmv_mexico_funds</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Bolsa Mexicana de Valores</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Mexican investment-fund listing and latest prices</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/es/Grupo_BMV/informacion-de-fondos</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/es/Grupo_BMV/informacion-de-fondos</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/es/Grupo_BMV/informacion-de-fondos</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Exchange public JSON</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Public registry / official website; programmatic access not yet confirmed</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Unknown — inspect source</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Candidate source</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>Usable Fund Data Confirmed</t>
+        </is>
+      </c>
+      <c r="Z7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>Integrated</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="n">
+        <v>5151</v>
+      </c>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bmv.com.mx/es/Grupo_BMV/informacion-de-fondos</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>Public BMV JSON lists operators, fund series, classifications by fund name, and latest price/NAV-like value for 5,151 series. Currency is normalized to MXN because the public price response does not publish a currency field; ISIN is not present. Capability notes: 5,151 fund/share-class identities; 3,670 latest price rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>cnbv_fund_statistics</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Comisión Nacional Bancaria y de Valores</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Investment fund statistical information</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gob.mx/cnbv/acciones-y-programas/informacion-estadistica-fondos-de-inversion</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gob.mx/cnbv/acciones-y-programas/informacion-estadistica-fondos-de-inversion</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gob.mx/cnbv/acciones-y-programas/informacion-estadistica-fondos-de-inversion</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Government regulator; statistical portal</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Public registry / official website; programmatic access not yet confirmed</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Unknown — inspect source</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Candidate source</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>Unavailable</t>
+        </is>
+      </c>
+      <c r="Z8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:55:49.331740+00:00</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr">
         <is>
           <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
         </is>
       </c>
-      <c r="AH5" s="2" t="inlineStr">
+      <c r="AH8" s="2" t="inlineStr">
         <is>
           <t>https://www.gob.mx/cnbv/acciones-y-programas/informacion-estadistica-fondos-de-inversion</t>
         </is>
       </c>
-      <c r="AI5" t="inlineStr">
+      <c r="AI8" t="inlineStr">
         <is>
           <t>Periodic fund-sector financial and operational series; granular downloadable format and reuse terms need checking. Capability notes: Fund aggregates; NAV not confirmed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AI5"/>
-  <conditionalFormatting sqref="Y2:Y5">
+  <autoFilter ref="A1:AI8"/>
+  <conditionalFormatting sqref="Y2:Y8">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>OR(Y2="Usable Fund Data Confirmed",Y2="Reachable")</formula>
     </cfRule>
@@ -5709,7 +6775,7 @@
       <formula>OR(Y2="Blocked",Y2="Unavailable")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA2:AA5">
+  <conditionalFormatting sqref="AA2:AA8">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AA2="Integrated"</formula>
     </cfRule>
@@ -5718,13 +6784,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="W2:W5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="W2:W8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Permitted,Restricted,Permission Required,Unknown"</formula1>
     </dataValidation>
-    <dataValidation sqref="Y2:Y5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Y2:Y8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Undiscovered,Discovered,Reachable,Authentication Required,Blocked,Unavailable,Accessible — No Fund Data,Usable Fund Data Confirmed"</formula1>
     </dataValidation>
-    <dataValidation sqref="AA2:AA5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AA2:AA8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,In Progress,Implemented,Tested,Integrated,Failed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5745,10 +6811,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH5" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH6" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH7" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH8" r:id="rId28"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId29"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6270,7 +7348,7 @@
       <c r="AD3" t="inlineStr"/>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="n">
-        <v>25678</v>
+        <v>37875</v>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
@@ -7557,7 +8635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7861,12 +8939,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>fca_authorised_funds</t>
+          <t>us_qqqm_etf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -7884,29 +8962,29 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>3975</v>
+        <v>1</v>
       </c>
       <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>cnbv_fund_statistics</t>
+          <t>scotia_canada_daily_nav</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Not implemented</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -7914,23 +8992,19 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+        <v>373</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>de_bde_nonmonetary_funds</t>
+          <t>bmv_mexico_funds</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -7948,19 +9022,19 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>6400</v>
+        <v>5151</v>
       </c>
       <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>amf_geco</t>
+          <t>uk_fundslibrary_unit_prices</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -7978,23 +9052,19 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>28375</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>finma_swiss_fund_list</t>
+          <t>uk_ft_morningstar_prices</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -8012,19 +9082,19 @@
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>2007</v>
+        <v>253</v>
       </c>
       <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>nl_bde_nonmonetary_funds</t>
+          <t>de_bundesanzeiger_navs</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>NL</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -8034,27 +9104,34 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Integrated</t>
+          <t>Failed</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>249</v>
       </c>
       <c r="G15" t="n">
-        <v>1306</v>
-      </c>
-      <c r="H15" t="inlineStr"/>
+        <v>127</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>ValidationError: 1 validation error for CanonicalNav
+nav
+  Input should be greater than 0 [type=greater_than, input_value='0.0', input_type=str]
+    For further information visit https://errors.pydantic.dev/2.14/v/greater_than</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>dk_bde_nonmonetary_funds</t>
+          <t>fca_authorised_funds</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DK</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -8072,19 +9149,19 @@
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>1486</v>
+        <v>3975</v>
       </c>
       <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>fi_fund_holdings</t>
+          <t>cnbv_fund_statistics</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -8113,12 +9190,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>lu_bde_nonmonetary_funds</t>
+          <t>de_bde_nonmonetary_funds</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>LU</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -8136,29 +9213,29 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>23955</v>
+        <v>6400</v>
       </c>
       <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cbI_fund_registers</t>
+          <t>amf_geco</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>IE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Not implemented</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -8166,7 +9243,7 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>28375</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -8177,12 +9254,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>it_bde_nonmonetary_funds</t>
+          <t>finma_swiss_fund_list</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -8200,29 +9277,29 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>1326</v>
+        <v>2007</v>
       </c>
       <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>imaj_fund_statistics</t>
+          <t>nl_bde_nonmonetary_funds</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>NL</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Not implemented</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -8230,23 +9307,19 @@
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+        <v>1306</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>csrc_public_fund_index</t>
+          <t>dk_bde_nonmonetary_funds</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>DK</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -8264,33 +9337,29 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>14170</v>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+        <v>1486</v>
+      </c>
+      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>gsfm_unit_prices</t>
+          <t>fi_fund_holdings</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Not implemented</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Integrated</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
@@ -8298,29 +9367,33 @@
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>1</v>
-      </c>
-      <c r="H23" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>kofia_fund_info</t>
+          <t>lu_bde_nonmonetary_funds</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>LU</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Not implemented</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
@@ -8328,23 +9401,19 @@
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+        <v>23955</v>
+      </c>
+      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>mas_opera_cis</t>
+          <t>cbI_fund_registers</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>IE</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -8373,12 +9442,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>hk_sfc_authorised_unit_trusts</t>
+          <t>it_bde_nonmonetary_funds</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>HK</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -8391,28 +9460,24 @@
           <t>Integrated</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>2026-10-18T19:45:12.781623+00:00</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="n">
-        <v>2255</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>2255</v>
+        <v>1326</v>
       </c>
       <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>sitca_fund_info</t>
+          <t>imaj_fund_statistics</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -8441,22 +9506,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>cbr_unit_fund_register</t>
+          <t>csrc_public_fund_index</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>CN</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Not implemented</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
@@ -8464,7 +9529,7 @@
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
+        <v>14170</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -8475,12 +9540,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>cvm_open_fund_data</t>
+          <t>gsfm_unit_prices</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -8498,33 +9563,29 @@
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>25678</v>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>uae_local_funds</t>
+          <t>au_user_managed_funds</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Not implemented</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -8532,33 +9593,29 @@
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+        <v>96</v>
+      </c>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>asisa_cis_fund_list</t>
+          <t>kofia_fund_info</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ZA</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Not implemented</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Integrated</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -8566,12 +9623,246 @@
         <v>0</v>
       </c>
       <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>mas_opera_cis</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Not implemented</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>hk_sfc_authorised_unit_trusts</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Integrated</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>2255</v>
+      </c>
+      <c r="H33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>sitca_fund_info</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Not implemented</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>cbr_unit_fund_register</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Not implemented</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>cvm_open_fund_data</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Integrated</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>37875</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>uae_local_funds</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Not implemented</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>asisa_cis_fund_list</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>ZA</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Integrated</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="n">
         <v>1945</v>
       </c>
-      <c r="H31" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H31"/>
+  <autoFilter ref="A1:H38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add Swiss SIX fund explorer NAV import
</commit_message>
<xml_diff>
--- a/reports/global_mutual_fund_source_inventory.xlsx
+++ b/reports/global_mutual_fund_source_inventory.xlsx
@@ -19,11 +19,11 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dashboard'!$A$1:$B$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Asia-Pacific'!$A$1:$AI$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Europe'!$A$1:$AI$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Europe'!$A$1:$AI$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'North America'!$A$1:$AI$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Other Markets'!$A$1:$AI$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Source Verification Log'!$A$1:$I$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'ETL Integration Status'!$A$1:$H$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'ETL Integration Status'!$A$1:$H$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Data Dictionary'!$A$1:$B$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -370,8 +370,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EuropeSources" displayName="EuropeSources" ref="A1:AI18" headerRowCount="1">
-  <autoFilter ref="A1:AI18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EuropeSources" displayName="EuropeSources" ref="A1:AI19" headerRowCount="1">
+  <autoFilter ref="A1:AI19"/>
   <tableColumns count="35">
     <tableColumn id="1" name="Source ID"/>
     <tableColumn id="2" name="Country"/>
@@ -850,7 +850,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7">
@@ -860,7 +860,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8">
@@ -870,7 +870,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9">
@@ -902,7 +902,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -2628,7 +2628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI18"/>
+  <dimension ref="A1:AI19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -3858,34 +3858,25 @@
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>Discovered</t>
+          <t>Usable Fund Data Confirmed</t>
         </is>
       </c>
       <c r="Z8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="n">
-        <v>249</v>
-      </c>
+      <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="n">
-        <v>127</v>
-      </c>
-      <c r="AG8" t="inlineStr">
-        <is>
-          <t>ValidationError: 1 validation error for CanonicalNav
-nav
-  Input should be greater than 0 [type=greater_than, input_value='0.0', input_type=str]
-    For further information visit https://errors.pydantic.dev/2.14/v/greater_than</t>
-        </is>
-      </c>
+        <v>248</v>
+      </c>
+      <c r="AG8" t="inlineStr"/>
       <c r="AH8" s="2" t="inlineStr">
         <is>
           <t>https://www.bundesanzeiger.de/pub/en/fondsdata</t>
@@ -3900,17 +3891,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>fca_authorised_funds</t>
+          <t>it_borsa_navs</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -3920,55 +3911,63 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Financial Conduct Authority</t>
+          <t>Borsa Italiana</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>UK authorised and recognised fund register</t>
+          <t>Daily NAV of open funds</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>https://www.fca.org.uk/freedom-information/information-consumer-investment-june-2026</t>
+          <t>https://www.borsaitaliana.it/fondi/fondi-aperti/nav/nav.en.htm</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>https://www.fca.org.uk/publication/fca/foi2026_01166-annex-a.csv</t>
+          <t>https://www.borsaitaliana.it/fondi/fondi-aperti/nav/nav.en.htm</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>https://www.fca.org.uk/freedom-information/information-consumer-investment-june-2026</t>
+          <t>https://www.borsaitaliana.it/fondi/fondi-aperti/nav/nav.en.htm</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Government regulator CSV snapshot</t>
+          <t>Exchange public NAV file</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Public FCA CSV download; no login</t>
-        </is>
-      </c>
-      <c r="L9" t="b">
-        <v>0</v>
+          <t>Public registry / official website; programmatic access not yet confirmed</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>CSV; Windows-1252; 11,842 product rows in the 2026-06 snapshot</t>
-        </is>
-      </c>
-      <c r="N9" t="b">
-        <v>1</v>
-      </c>
-      <c r="O9" t="b">
-        <v>0</v>
-      </c>
-      <c r="P9" t="b">
-        <v>0</v>
+          <t>Unknown — inspect source</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Candidate source</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -3977,22 +3976,22 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>FCA Product Reference Number (PRN)</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Snapshot published 2026-06-24</t>
+          <t>Not confirmed</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Snapshot publication; refresh when FCA posts a new file</t>
+          <t>Not confirmed</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -4007,7 +4006,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>Unknown — confirm FCA reuse terms</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
@@ -4024,38 +4023,48 @@
         </is>
       </c>
       <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr"/>
-      <c r="AD9" t="inlineStr"/>
-      <c r="AE9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>2026-10-26T10:29:47.007586+00:00</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>2026-10-26T10:29:47.007586+00:00</t>
+        </is>
+      </c>
+      <c r="AE9" t="n">
+        <v>68</v>
+      </c>
       <c r="AF9" t="n">
-        <v>3975</v>
+        <v>68</v>
       </c>
       <c r="AG9" t="inlineStr"/>
       <c r="AH9" s="2" t="inlineStr">
         <is>
-          <t>https://www.fca.org.uk/freedom-information/information-consumer-investment-june-2026</t>
+          <t>https://www.borsaitaliana.it/fondi/fondi-aperti/nav/nav.en.htm</t>
         </is>
       </c>
       <c r="AI9" t="inlineStr">
         <is>
-          <t>Imported rows are limited to FCA statuses Authorised and Approved, which FCA identifies as UK-domiciled. Recognised offshore rows are excluded. Currency and NAV remain null/not loaded.</t>
+          <t>Borsa Italiana publishes a free daily text file for all open funds with reference date, ISIN, NAV currency, NAV and NAV in euro. This snapshot produced 68 validated observations. The daily text file does not publish fund names or categories, so names are ISIN-labelled and category is explicitly marked unavailable; the existing BDE Italy connector remains the broader 1,326-fund identity master. Capability notes: 68 daily NAV observations with ISIN and EUR/foreign currency</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>de_bde_nonmonetary_funds</t>
+          <t>fca_authorised_funds</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -4065,37 +4074,37 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Banco de España</t>
+          <t>Financial Conduct Authority</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>List of non-monetary investment funds in Germany</t>
+          <t>UK authorised and recognised fund register</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-de.html</t>
+          <t>https://www.fca.org.uk/freedom-information/information-consumer-investment-june-2026</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-de.csv</t>
+          <t>https://www.fca.org.uk/publication/fca/foi2026_01166-annex-a.csv</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-de.html</t>
+          <t>https://www.fca.org.uk/freedom-information/information-consumer-investment-june-2026</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Official statistical fund register CSV</t>
+          <t>Government regulator CSV snapshot</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Public Banco de España country-level CSV; no login</t>
+          <t>Public FCA CSV download; no login</t>
         </is>
       </c>
       <c r="L10" t="b">
@@ -4103,7 +4112,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>UTF-8 CSV; fund code, LEI, name, manager, address, policy and open/closed status</t>
+          <t>CSV; Windows-1252; 11,842 product rows in the 2026-06 snapshot</t>
         </is>
       </c>
       <c r="N10" t="b">
@@ -4127,17 +4136,17 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>European code; LEI where present</t>
+          <t>FCA Product Reference Number (PRN)</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Current fund-register snapshot</t>
+          <t>Snapshot published 2026-06-24</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Snapshot; check for updates</t>
+          <t>Snapshot publication; refresh when FCA posts a new file</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -4152,7 +4161,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>Unknown — confirm Banco de España reuse terms</t>
+          <t>Unknown — confirm FCA reuse terms</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
@@ -4173,34 +4182,34 @@
       <c r="AD10" t="inlineStr"/>
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="n">
-        <v>6400</v>
+        <v>3975</v>
       </c>
       <c r="AG10" t="inlineStr"/>
       <c r="AH10" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-de.html</t>
+          <t>https://www.fca.org.uk/freedom-information/information-consumer-investment-june-2026</t>
         </is>
       </c>
       <c r="AI10" t="inlineStr">
         <is>
-          <t>Imports only open-ended non-monetary investment fund entries for this domicile. Register includes UCITS and AIF categories; it is broader than a strict UCITS-only universe. No NAV or currency is inferred.</t>
+          <t>Imported rows are limited to FCA statuses Authorised and Approved, which FCA identifies as UK-domiciled. Recognised offshore rows are excluded. Currency and NAV remain null/not loaded.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>amf_geco</t>
+          <t>de_bde_nonmonetary_funds</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -4210,37 +4219,37 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Autorité des marchés financiers</t>
+          <t>Banco de España</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>GECO French-domiciled OPC product/share-class export</t>
+          <t>List of non-monetary investment funds in Germany</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>https://geco.amf-france.org/liste-des-produits-d-epargne</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-de.html</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>https://geco.amf-france.org/back-office/funds/compartments</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-de.csv</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>https://geco.amf-france.org/liste-des-produits-d-epargne</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-de.html</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Government regulator JSON export</t>
+          <t>Official statistical fund register CSV</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Public AMF GECO JSON export using the web client request format</t>
+          <t>Public Banco de España country-level CSV; no login</t>
         </is>
       </c>
       <c r="L11" t="b">
@@ -4248,7 +4257,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>JSON; product and compartment/share-class records</t>
+          <t>UTF-8 CSV; fund code, LEI, name, manager, address, policy and open/closed status</t>
         </is>
       </c>
       <c r="N11" t="b">
@@ -4267,22 +4276,22 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>None in this export</t>
+          <t>None</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>AMF compartment ID, AMF product ID and ISIN where present</t>
+          <t>European code; LEI where present</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Current active product snapshot; no NAV history</t>
+          <t>Current fund-register snapshot</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Current export on demand</t>
+          <t>Snapshot; check for updates</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -4297,7 +4306,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>Unknown — confirm AMF reuse terms</t>
+          <t>Unknown — confirm Banco de España reuse terms</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
@@ -4314,46 +4323,38 @@
         </is>
       </c>
       <c r="AB11" t="inlineStr"/>
-      <c r="AC11" t="inlineStr">
-        <is>
-          <t>2026-10-17T11:55:49.437058+00:00</t>
-        </is>
-      </c>
+      <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr"/>
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="n">
-        <v>28375</v>
-      </c>
-      <c r="AG11" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+        <v>6400</v>
+      </c>
+      <c r="AG11" t="inlineStr"/>
       <c r="AH11" s="2" t="inlineStr">
         <is>
-          <t>https://geco.amf-france.org/liste-des-produits-d-epargne</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-de.html</t>
         </is>
       </c>
       <c r="AI11" t="inlineStr">
         <is>
-          <t>ETL filters active French-domiciled products and expands available share-class ISINs. Foreign-domiciled products authorised for marketing in France are excluded. No currency or NAV is inferred.</t>
+          <t>Imports only open-ended non-monetary investment fund entries for this domicile. Register includes UCITS and AIF categories; it is broader than a strict UCITS-only universe. No NAV or currency is inferred.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>finma_swiss_fund_list</t>
+          <t>amf_geco</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -4363,37 +4364,37 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Swiss Financial Market Supervisory Authority</t>
+          <t>Autorité des marchés financiers</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Approved Swiss collective investment schemes</t>
+          <t>GECO French-domiciled OPC product/share-class export</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>https://www.finma.ch/en/finma-public/authorised-institutions-individuals-and-products/</t>
+          <t>https://geco.amf-france.org/liste-des-produits-d-epargne</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>https://www.finma.ch/~/media/finma/dokumente/bewilligungstraeger/pdf/afch.pdf?la=en%3BApproved</t>
+          <t>https://geco.amf-france.org/back-office/funds/compartments</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>https://www.finma.ch/en/finma-public/authorised-institutions-individuals-and-products/</t>
+          <t>https://geco.amf-france.org/liste-des-produits-d-epargne</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Government regulator PDF</t>
+          <t>Government regulator JSON export</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Public FINMA PDF download; no login</t>
+          <t>Public AMF GECO JSON export using the web client request format</t>
         </is>
       </c>
       <c r="L12" t="b">
@@ -4401,7 +4402,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>PDF; tabular list with individual fund name and FINMA-ID</t>
+          <t>JSON; product and compartment/share-class records</t>
         </is>
       </c>
       <c r="N12" t="b">
@@ -4420,22 +4421,22 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>None in approved-funds list</t>
+          <t>None in this export</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>FINMA-ID</t>
+          <t>AMF compartment ID, AMF product ID and ISIN where present</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Current approved-funds list, dated 2026-10-18</t>
+          <t>Current active product snapshot; no NAV history</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>FINMA republishes the register periodically</t>
+          <t>Current export on demand</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
@@ -4450,7 +4451,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>Unknown — confirm FINMA reuse terms</t>
+          <t>Unknown — confirm AMF reuse terms</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
@@ -4467,38 +4468,46 @@
         </is>
       </c>
       <c r="AB12" t="inlineStr"/>
-      <c r="AC12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:55:49.437058+00:00</t>
+        </is>
+      </c>
       <c r="AD12" t="inlineStr"/>
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="n">
-        <v>2007</v>
-      </c>
-      <c r="AG12" t="inlineStr"/>
+        <v>28375</v>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
       <c r="AH12" s="2" t="inlineStr">
         <is>
-          <t>https://www.finma.ch/en/finma-public/authorised-institutions-individuals-and-products/</t>
+          <t>https://geco.amf-france.org/liste-des-produits-d-epargne</t>
         </is>
       </c>
       <c r="AI12" t="inlineStr">
         <is>
-          <t>The FINMA domestic approved-schemes PDF has individual fund/sub-fund names and FINMA IDs. The connector imports those product rows; it does not infer currency or NAV.</t>
+          <t>ETL filters active French-domiciled products and expands available share-class ISINs. Foreign-domiciled products authorised for marketing in France are excluded. No currency or NAV is inferred.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>nl_bde_nonmonetary_funds</t>
+          <t>finma_swiss_fund_list</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>NL</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -4508,37 +4517,37 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Banco de España</t>
+          <t>Swiss Financial Market Supervisory Authority</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>List of non-monetary investment funds in the Netherlands</t>
+          <t>Approved Swiss collective investment schemes</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-nl.html</t>
+          <t>https://www.finma.ch/en/finma-public/authorised-institutions-individuals-and-products/</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-nl.csv</t>
+          <t>https://www.finma.ch/~/media/finma/dokumente/bewilligungstraeger/pdf/afch.pdf?la=en%3BApproved</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-nl.html</t>
+          <t>https://www.finma.ch/en/finma-public/authorised-institutions-individuals-and-products/</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Official statistical fund register CSV</t>
+          <t>Government regulator PDF</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Public Banco de España country-level CSV; no login</t>
+          <t>Public FINMA PDF download; no login</t>
         </is>
       </c>
       <c r="L13" t="b">
@@ -4546,7 +4555,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>UTF-8 CSV; fund code, LEI, name, manager, address, policy and open/closed status</t>
+          <t>PDF; tabular list with individual fund name and FINMA-ID</t>
         </is>
       </c>
       <c r="N13" t="b">
@@ -4565,22 +4574,22 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None in approved-funds list</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>European code; LEI where present</t>
+          <t>FINMA-ID</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Current fund-register snapshot</t>
+          <t>Current approved-funds list, dated 2026-10-18</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Snapshot; check for updates</t>
+          <t>FINMA republishes the register periodically</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
@@ -4595,7 +4604,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>Unknown — confirm Banco de España reuse terms</t>
+          <t>Unknown — confirm FINMA reuse terms</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
@@ -4616,34 +4625,34 @@
       <c r="AD13" t="inlineStr"/>
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="n">
-        <v>1306</v>
+        <v>2007</v>
       </c>
       <c r="AG13" t="inlineStr"/>
       <c r="AH13" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-nl.html</t>
+          <t>https://www.finma.ch/en/finma-public/authorised-institutions-individuals-and-products/</t>
         </is>
       </c>
       <c r="AI13" t="inlineStr">
         <is>
-          <t>Imports only open-ended non-monetary investment fund entries for this domicile. Register includes UCITS and AIF categories; it is broader than a strict UCITS-only universe. No NAV or currency is inferred.</t>
+          <t>The FINMA domestic approved-schemes PDF has individual fund/sub-fund names and FINMA IDs. The connector imports those product rows; it does not infer currency or NAV.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>dk_bde_nonmonetary_funds</t>
+          <t>nl_bde_nonmonetary_funds</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>DK</t>
+          <t>NL</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -4658,32 +4667,32 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>List of non-monetary investment funds in Denmark</t>
+          <t>List of non-monetary investment funds in the Netherlands</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-dk.html</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-nl.html</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-dk.csv</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-nl.csv</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-dk.html</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-nl.html</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Official national statistical register CSV</t>
+          <t>Official statistical fund register CSV</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Public CSV download; no login</t>
+          <t>Public Banco de España country-level CSV; no login</t>
         </is>
       </c>
       <c r="L14" t="b">
@@ -4691,7 +4700,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>CSV; UTF-8; seven published columns plus an empty padded column</t>
+          <t>UTF-8 CSV; fund code, LEI, name, manager, address, policy and open/closed status</t>
         </is>
       </c>
       <c r="N14" t="b">
@@ -4715,17 +4724,17 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>European code, LEI where present</t>
+          <t>European code; LEI where present</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Current register snapshot</t>
+          <t>Current fund-register snapshot</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Register snapshot; check source for updates</t>
+          <t>Snapshot; check for updates</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
@@ -4761,34 +4770,34 @@
       <c r="AD14" t="inlineStr"/>
       <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="n">
-        <v>1486</v>
+        <v>1306</v>
       </c>
       <c r="AG14" t="inlineStr"/>
       <c r="AH14" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-dk.html</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-nl.html</t>
         </is>
       </c>
       <c r="AI14" t="inlineStr">
         <is>
-          <t>Imports open-ended Danish non-monetary investment funds only. The source also includes AIFs, so this is broader than a strict UCITS mutual-fund universe. No currency or NAV is inferred.</t>
+          <t>Imports only open-ended non-monetary investment fund entries for this domicile. Register includes UCITS and AIF categories; it is broader than a strict UCITS-only universe. No NAV or currency is inferred.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>fi_fund_holdings</t>
+          <t>dk_bde_nonmonetary_funds</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>DK</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -4798,63 +4807,55 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Finansinspektionen</t>
+          <t>Banco de España</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Fund holdings register</t>
+          <t>List of non-monetary investment funds in Denmark</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>https://www.fi.se/en/our-registers/fund-holdings/</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-dk.html</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>https://www.fi.se/en/our-registers/fund-holdings/</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-dk.csv</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>https://www.fi.se/en/our-registers/fund-holdings/</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-dk.html</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Government regulator reporting data</t>
+          <t>Official national statistical register CSV</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Public registry / official website; programmatic access not yet confirmed</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
+          <t>Public CSV download; no login</t>
+        </is>
+      </c>
+      <c r="L15" t="b">
+        <v>0</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Unknown — inspect source</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Candidate source</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
+          <t>CSV; UTF-8; seven published columns plus an empty padded column</t>
+        </is>
+      </c>
+      <c r="N15" t="b">
+        <v>1</v>
+      </c>
+      <c r="O15" t="b">
+        <v>0</v>
+      </c>
+      <c r="P15" t="b">
+        <v>0</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -4863,29 +4864,29 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>None</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>European code, LEI where present</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
+          <t>Current register snapshot</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Register snapshot; check source for updates</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
           <t>Not confirmed</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>Not confirmed</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>Not confirmed</t>
-        </is>
-      </c>
       <c r="W15" t="inlineStr">
         <is>
           <t>Unknown</t>
@@ -4893,61 +4894,55 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Unknown — confirm Banco de España reuse terms</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>Unavailable</t>
+          <t>Usable Fund Data Confirmed</t>
         </is>
       </c>
       <c r="Z15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr"/>
-      <c r="AC15" t="inlineStr">
-        <is>
-          <t>2026-10-17T11:55:49.651051+00:00</t>
-        </is>
-      </c>
+      <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="inlineStr"/>
       <c r="AE15" t="inlineStr"/>
-      <c r="AF15" t="inlineStr"/>
-      <c r="AG15" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+      <c r="AF15" t="n">
+        <v>1486</v>
+      </c>
+      <c r="AG15" t="inlineStr"/>
       <c r="AH15" s="2" t="inlineStr">
         <is>
-          <t>https://www.fi.se/en/our-registers/fund-holdings/</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-dk.html</t>
         </is>
       </c>
       <c r="AI15" t="inlineStr">
         <is>
-          <t>FI publishes fund holdings data; special-fund holdings are excluded. This supports holdings research, not fund NAV coverage. Capability notes: Fund holdings; NAV not confirmed</t>
+          <t>Imports open-ended Danish non-monetary investment funds only. The source also includes AIFs, so this is broader than a strict UCITS mutual-fund universe. No currency or NAV is inferred.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>lu_bde_nonmonetary_funds</t>
+          <t>fi_fund_holdings</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>LU</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -4957,55 +4952,63 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Banco de España</t>
+          <t>Finansinspektionen</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>List of non-monetary investment funds in Luxembourg</t>
+          <t>Fund holdings register</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-lu.html</t>
+          <t>https://www.fi.se/en/our-registers/fund-holdings/</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-lu.csv</t>
+          <t>https://www.fi.se/en/our-registers/fund-holdings/</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-lu.html</t>
+          <t>https://www.fi.se/en/our-registers/fund-holdings/</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Official statistical fund register CSV</t>
+          <t>Government regulator reporting data</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Public Banco de España country-level CSV; no login</t>
-        </is>
-      </c>
-      <c r="L16" t="b">
-        <v>0</v>
+          <t>Public registry / official website; programmatic access not yet confirmed</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>UTF-8 CSV; fund code, LEI, name, manager, address, policy and open/closed status</t>
-        </is>
-      </c>
-      <c r="N16" t="b">
-        <v>1</v>
-      </c>
-      <c r="O16" t="b">
-        <v>0</v>
-      </c>
-      <c r="P16" t="b">
-        <v>0</v>
+          <t>Unknown — inspect source</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Candidate source</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -5014,22 +5017,22 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>European code; LEI where present</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Current fund-register snapshot</t>
+          <t>Not confirmed</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>Snapshot; check for updates</t>
+          <t>Not confirmed</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
@@ -5044,55 +5047,61 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>Unknown — confirm Banco de España reuse terms</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>Usable Fund Data Confirmed</t>
+          <t>Unavailable</t>
         </is>
       </c>
       <c r="Z16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>Integrated</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr"/>
-      <c r="AC16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:55:49.651051+00:00</t>
+        </is>
+      </c>
       <c r="AD16" t="inlineStr"/>
       <c r="AE16" t="inlineStr"/>
-      <c r="AF16" t="n">
-        <v>23955</v>
-      </c>
-      <c r="AG16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr"/>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
       <c r="AH16" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-lu.html</t>
+          <t>https://www.fi.se/en/our-registers/fund-holdings/</t>
         </is>
       </c>
       <c r="AI16" t="inlineStr">
         <is>
-          <t>Imports only open-ended non-monetary investment fund entries for this domicile. Register includes UCITS and AIF categories; it is broader than a strict UCITS-only universe. No NAV or currency is inferred.</t>
+          <t>FI publishes fund holdings data; special-fund holdings are excluded. This supports holdings research, not fund NAV coverage. Capability notes: Fund holdings; NAV not confirmed</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>cbI_fund_registers</t>
+          <t>lu_bde_nonmonetary_funds</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>IE</t>
+          <t>LU</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -5102,63 +5111,55 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Central Bank of Ireland</t>
+          <t>Banco de España</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Collective investment scheme registers and downloads</t>
+          <t>List of non-monetary investment funds in Luxembourg</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>https://registers.centralbank.ie/downloadspage.aspx</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-lu.html</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>https://registers.centralbank.ie/downloadspage.aspx</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-lu.csv</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>https://registers.centralbank.ie/downloadspage.aspx</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-lu.html</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Government regulator register and downloads</t>
+          <t>Official statistical fund register CSV</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Public registry / official website; programmatic access not yet confirmed</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
+          <t>Public Banco de España country-level CSV; no login</t>
+        </is>
+      </c>
+      <c r="L17" t="b">
+        <v>0</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Unknown — inspect source</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Candidate source</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
+          <t>UTF-8 CSV; fund code, LEI, name, manager, address, policy and open/closed status</t>
+        </is>
+      </c>
+      <c r="N17" t="b">
+        <v>1</v>
+      </c>
+      <c r="O17" t="b">
+        <v>0</v>
+      </c>
+      <c r="P17" t="b">
+        <v>0</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -5167,29 +5168,29 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>None</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>European code; LEI where present</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
+          <t>Current fund-register snapshot</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Snapshot; check for updates</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
           <t>Not confirmed</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>Not confirmed</t>
-        </is>
-      </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>Not confirmed</t>
-        </is>
-      </c>
       <c r="W17" t="inlineStr">
         <is>
           <t>Unknown</t>
@@ -5197,61 +5198,55 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Unknown — confirm Banco de España reuse terms</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>Unavailable</t>
+          <t>Usable Fund Data Confirmed</t>
         </is>
       </c>
       <c r="Z17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="AB17" t="inlineStr"/>
-      <c r="AC17" t="inlineStr">
-        <is>
-          <t>2026-10-17T11:55:49.758179+00:00</t>
-        </is>
-      </c>
+      <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="inlineStr"/>
       <c r="AE17" t="inlineStr"/>
-      <c r="AF17" t="inlineStr"/>
-      <c r="AG17" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+      <c r="AF17" t="n">
+        <v>23955</v>
+      </c>
+      <c r="AG17" t="inlineStr"/>
       <c r="AH17" s="2" t="inlineStr">
         <is>
-          <t>https://registers.centralbank.ie/downloadspage.aspx</t>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-lu.html</t>
         </is>
       </c>
       <c r="AI17" t="inlineStr">
         <is>
-          <t>Official CIS search and downloads include authorised funds and UCITS lists, generally PDF; monthly fund-data publications are available, format suitability needs inspection. Capability notes: Fund master; monthly fund reports</t>
+          <t>Imports only open-ended non-monetary investment fund entries for this domicile. Register includes UCITS and AIF categories; it is broader than a strict UCITS-only universe. No NAV or currency is inferred.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>it_bde_nonmonetary_funds</t>
+          <t>cbI_fund_registers</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>IE</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -5261,55 +5256,63 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Banco de España</t>
+          <t>Central Bank of Ireland</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>List of non-monetary investment funds in Italy</t>
+          <t>Collective investment scheme registers and downloads</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-it.html</t>
+          <t>https://registers.centralbank.ie/downloadspage.aspx</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-it.csv</t>
+          <t>https://registers.centralbank.ie/downloadspage.aspx</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-it.html</t>
+          <t>https://registers.centralbank.ie/downloadspage.aspx</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Official statistical fund register CSV</t>
+          <t>Government regulator register and downloads</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Public Banco de España country-level CSV; no login</t>
-        </is>
-      </c>
-      <c r="L18" t="b">
-        <v>0</v>
+          <t>Public registry / official website; programmatic access not yet confirmed</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>UTF-8 CSV; fund code, LEI, name, manager, address, policy and open/closed status</t>
-        </is>
-      </c>
-      <c r="N18" t="b">
-        <v>1</v>
-      </c>
-      <c r="O18" t="b">
-        <v>0</v>
-      </c>
-      <c r="P18" t="b">
-        <v>0</v>
+          <t>Unknown — inspect source</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Candidate source</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -5318,22 +5321,22 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>European code; LEI where present</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Current fund-register snapshot</t>
+          <t>Not confirmed</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>Snapshot; check for updates</t>
+          <t>Not confirmed</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
@@ -5348,44 +5351,195 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>Unknown — confirm Banco de España reuse terms</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>Usable Fund Data Confirmed</t>
+          <t>Unavailable</t>
         </is>
       </c>
       <c r="Z18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>Integrated</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="AB18" t="inlineStr"/>
-      <c r="AC18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:55:49.758179+00:00</t>
+        </is>
+      </c>
       <c r="AD18" t="inlineStr"/>
       <c r="AE18" t="inlineStr"/>
-      <c r="AF18" t="n">
+      <c r="AF18" t="inlineStr"/>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
+      <c r="AH18" s="2" t="inlineStr">
+        <is>
+          <t>https://registers.centralbank.ie/downloadspage.aspx</t>
+        </is>
+      </c>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>Official CIS search and downloads include authorised funds and UCITS lists, generally PDF; monthly fund-data publications are available, format suitability needs inspection. Capability notes: Fund master; monthly fund reports</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>it_bde_nonmonetary_funds</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Banco de España</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>List of non-monetary investment funds in Italy</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-it.html</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-it.csv</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-it.html</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Official statistical fund register CSV</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Public Banco de España country-level CSV; no login</t>
+        </is>
+      </c>
+      <c r="L19" t="b">
+        <v>0</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>UTF-8 CSV; fund code, LEI, name, manager, address, policy and open/closed status</t>
+        </is>
+      </c>
+      <c r="N19" t="b">
+        <v>1</v>
+      </c>
+      <c r="O19" t="b">
+        <v>0</v>
+      </c>
+      <c r="P19" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>European code; LEI where present</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Current fund-register snapshot</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Snapshot; check for updates</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>Not confirmed</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>Unknown — confirm Banco de España reuse terms</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>Usable Fund Data Confirmed</t>
+        </is>
+      </c>
+      <c r="Z19" t="b">
+        <v>1</v>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>Integrated</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
+      <c r="AD19" t="inlineStr"/>
+      <c r="AE19" t="inlineStr"/>
+      <c r="AF19" t="n">
         <v>1326</v>
       </c>
-      <c r="AG18" t="inlineStr"/>
-      <c r="AH18" s="2" t="inlineStr">
+      <c r="AG19" t="inlineStr"/>
+      <c r="AH19" s="2" t="inlineStr">
         <is>
           <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/clasificacion-entidades/listas-instituciones-financieras/listas-fondos-inversion-pais/lista-if-it.html</t>
         </is>
       </c>
-      <c r="AI18" t="inlineStr">
+      <c r="AI19" t="inlineStr">
         <is>
           <t>Imports only open-ended non-monetary investment fund entries for this domicile. Register includes UCITS and AIF categories; it is broader than a strict UCITS-only universe. No NAV or currency is inferred.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AI18"/>
-  <conditionalFormatting sqref="Y2:Y18">
+  <autoFilter ref="A1:AI19"/>
+  <conditionalFormatting sqref="Y2:Y19">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>OR(Y2="Usable Fund Data Confirmed",Y2="Reachable")</formula>
     </cfRule>
@@ -5393,7 +5547,7 @@
       <formula>OR(Y2="Blocked",Y2="Unavailable")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA2:AA18">
+  <conditionalFormatting sqref="AA2:AA19">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AA2="Integrated"</formula>
     </cfRule>
@@ -5402,13 +5556,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="W2:W18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="W2:W19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Permitted,Restricted,Permission Required,Unknown"</formula1>
     </dataValidation>
-    <dataValidation sqref="Y2:Y18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Y2:Y19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Undiscovered,Discovered,Reachable,Authentication Required,Blocked,Unavailable,Accessible — No Fund Data,Usable Fund Data Confirmed"</formula1>
     </dataValidation>
-    <dataValidation sqref="AA2:AA18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AA2:AA19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,In Progress,Implemented,Tested,Integrated,Failed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5481,10 +5635,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH18" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AH19" r:id="rId72"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId69"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId73"/>
   </tableParts>
 </worksheet>
 </file>
@@ -8635,7 +8793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9104,34 +9262,27 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="n">
-        <v>249</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>127</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>ValidationError: 1 validation error for CanonicalNav
-nav
-  Input should be greater than 0 [type=greater_than, input_value='0.0', input_type=str]
-    For further information visit https://errors.pydantic.dev/2.14/v/greater_than</t>
-        </is>
-      </c>
+        <v>248</v>
+      </c>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>fca_authorised_funds</t>
+          <t>it_borsa_navs</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -9144,34 +9295,38 @@
           <t>Integrated</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-10-26T10:29:47.007586+00:00</t>
+        </is>
+      </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="G16" t="n">
-        <v>3975</v>
+        <v>68</v>
       </c>
       <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>cnbv_fund_statistics</t>
+          <t>fca_authorised_funds</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Not implemented</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -9179,33 +9334,29 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+        <v>3975</v>
+      </c>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>de_bde_nonmonetary_funds</t>
+          <t>cnbv_fund_statistics</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Not implemented</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Integrated</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -9213,19 +9364,23 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>6400</v>
-      </c>
-      <c r="H18" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>amf_geco</t>
+          <t>de_bde_nonmonetary_funds</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -9243,23 +9398,19 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>28375</v>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+        <v>6400</v>
+      </c>
+      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>finma_swiss_fund_list</t>
+          <t>amf_geco</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -9277,19 +9428,23 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>2007</v>
-      </c>
-      <c r="H20" t="inlineStr"/>
+        <v>28375</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>nl_bde_nonmonetary_funds</t>
+          <t>finma_swiss_fund_list</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>NL</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -9307,19 +9462,19 @@
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>1306</v>
+        <v>2007</v>
       </c>
       <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>dk_bde_nonmonetary_funds</t>
+          <t>nl_bde_nonmonetary_funds</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DK</t>
+          <t>NL</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -9337,29 +9492,29 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>1486</v>
+        <v>1306</v>
       </c>
       <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>fi_fund_holdings</t>
+          <t>dk_bde_nonmonetary_funds</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>DK</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Not implemented</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
@@ -9367,33 +9522,29 @@
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+        <v>1486</v>
+      </c>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>lu_bde_nonmonetary_funds</t>
+          <t>fi_fund_holdings</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>LU</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Not implemented</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Integrated</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
@@ -9401,29 +9552,33 @@
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>23955</v>
-      </c>
-      <c r="H24" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>cbI_fund_registers</t>
+          <t>lu_bde_nonmonetary_funds</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>IE</t>
+          <t>LU</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Not implemented</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
@@ -9431,33 +9586,29 @@
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+        <v>23955</v>
+      </c>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>it_bde_nonmonetary_funds</t>
+          <t>cbI_fund_registers</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>IE</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Not implemented</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Integrated</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
@@ -9465,29 +9616,33 @@
         <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>1326</v>
-      </c>
-      <c r="H26" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>imaj_fund_statistics</t>
+          <t>it_bde_nonmonetary_funds</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Not implemented</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
@@ -9495,33 +9650,29 @@
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+        <v>1326</v>
+      </c>
+      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>csrc_public_fund_index</t>
+          <t>imaj_fund_statistics</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Not implemented</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Integrated</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
@@ -9529,7 +9680,7 @@
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>14170</v>
+        <v>0</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -9540,12 +9691,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>gsfm_unit_prices</t>
+          <t>csrc_public_fund_index</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>CN</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -9563,14 +9714,18 @@
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>1</v>
-      </c>
-      <c r="H29" t="inlineStr"/>
+        <v>14170</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>au_user_managed_funds</t>
+          <t>gsfm_unit_prices</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -9593,29 +9748,29 @@
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>96</v>
+        <v>1</v>
       </c>
       <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>kofia_fund_info</t>
+          <t>au_user_managed_funds</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Not implemented</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -9623,23 +9778,19 @@
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+        <v>96</v>
+      </c>
+      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>mas_opera_cis</t>
+          <t>kofia_fund_info</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -9668,22 +9819,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>hk_sfc_authorised_unit_trusts</t>
+          <t>mas_opera_cis</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>HK</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Not implemented</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Integrated</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -9691,29 +9842,33 @@
         <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>2255</v>
-      </c>
-      <c r="H33" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>sitca_fund_info</t>
+          <t>hk_sfc_authorised_unit_trusts</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>HK</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Not implemented</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -9721,23 +9876,19 @@
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
-        </is>
-      </c>
+        <v>2255</v>
+      </c>
+      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>cbr_unit_fund_register</t>
+          <t>sitca_fund_info</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>RU</t>
+          <t>TW</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -9766,22 +9917,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>cvm_open_fund_data</t>
+          <t>cbr_unit_fund_register</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>RU</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Not implemented</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Integrated</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -9789,7 +9940,7 @@
         <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>37875</v>
+        <v>0</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -9800,22 +9951,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>uae_local_funds</t>
+          <t>cvm_open_fund_data</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Not implemented</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
@@ -9823,7 +9974,7 @@
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>0</v>
+        <v>37875</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -9834,22 +9985,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>asisa_cis_fund_list</t>
+          <t>uae_local_funds</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ZA</t>
+          <t>AE</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Implemented</t>
+          <t>Not implemented</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Integrated</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
@@ -9857,12 +10008,46 @@
         <v>0</v>
       </c>
       <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>ConnectError: [Errno -3] Temporary failure in name resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>asisa_cis_fund_list</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ZA</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Integrated</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
         <v>1945</v>
       </c>
-      <c r="H38" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H38"/>
+  <autoFilter ref="A1:H39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>